<commit_message>
UI strings QA sheet: skip-penalty option is just "Yes" (owner edit)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CharaDUO-UI-strings.xlsx
+++ b/CharaDUO-UI-strings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ryopang/Documents/Claude Code/Project DUO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D680AC9-31DF-CA49-AF5A-A854B1A2D11C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E721415C-3154-B744-A8AB-CB533BFC62BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="351">
   <si>
     <t>key</t>
   </si>
@@ -971,9 +971,6 @@
   </si>
   <si>
     <t>While a round is running, the guessing team is filmed and the table is recorded with sound — so the describer's voice is captured too.</t>
-  </si>
-  <si>
-    <t>Yes (−1)</t>
   </si>
   <si>
     <t>You can turn the camera off any time in Settings. The game plays fine without it.</t>
@@ -1851,10 +1848,10 @@
         <v>80</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>81</v>
@@ -1868,7 +1865,7 @@
         <v>82</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>83</v>
@@ -2002,7 +1999,7 @@
         <v>111</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>112</v>
@@ -2130,13 +2127,13 @@
         <v>131</v>
       </c>
       <c r="C38" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="D38" s="1" t="s">
         <v>330</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="E38" s="1" t="s">
         <v>331</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>332</v>
       </c>
       <c r="F38" s="1" t="s">
         <v>132</v>
@@ -2442,7 +2439,7 @@
         <v>194</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D56" s="1" t="s">
         <v>195</v>
@@ -2553,13 +2550,13 @@
         <v>212</v>
       </c>
       <c r="C62" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="E62" s="1" t="s">
         <v>334</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>334</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="63" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -2570,13 +2567,13 @@
         <v>213</v>
       </c>
       <c r="C63" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="E63" s="1" t="s">
         <v>334</v>
-      </c>
-      <c r="D63" s="1" t="s">
-        <v>334</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="64" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -2587,13 +2584,13 @@
         <v>214</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F64" s="1" t="s">
         <v>215</v>
@@ -2661,13 +2658,13 @@
         <v>227</v>
       </c>
       <c r="C68" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="E68" s="1" t="s">
         <v>339</v>
-      </c>
-      <c r="D68" s="1" t="s">
-        <v>339</v>
-      </c>
-      <c r="E68" s="1" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -2698,10 +2695,10 @@
         <v>232</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="71" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -2715,10 +2712,10 @@
         <v>234</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="72" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -3036,16 +3033,16 @@
         <v>292</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C89" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="D89" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="D89" s="1" t="s">
+      <c r="E89" s="1" t="s">
         <v>342</v>
-      </c>
-      <c r="E89" s="1" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="90" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -3053,7 +3050,7 @@
         <v>293</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C90" s="1" t="s">
         <v>294</v>
@@ -3158,16 +3155,16 @@
         <v>316</v>
       </c>
       <c r="B96" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="C96" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="C96" s="1" t="s">
+      <c r="D96" s="1" t="s">
         <v>347</v>
       </c>
-      <c r="D96" s="1" t="s">
+      <c r="E96" s="1" t="s">
         <v>348</v>
-      </c>
-      <c r="E96" s="1" t="s">
-        <v>349</v>
       </c>
       <c r="F96" s="1" t="s">
         <v>85</v>
@@ -3175,36 +3172,36 @@
     </row>
     <row r="97" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
-        <v>317</v>
+        <v>349</v>
       </c>
       <c r="B97" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="C97" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="C97" s="1" t="s">
-        <v>351</v>
-      </c>
       <c r="D97" s="1" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="98" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="C98" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="B98" s="1" t="s">
-        <v>318</v>
-      </c>
-      <c r="C98" s="1" t="s">
+      <c r="D98" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="D98" s="1" t="s">
+      <c r="E98" s="1" t="s">
         <v>320</v>
-      </c>
-      <c r="E98" s="1" t="s">
-        <v>321</v>
       </c>
       <c r="F98" s="1" t="s">
         <v>85</v>

</xml_diff>